<commit_message>
Add FastAPI services and desktop migration
</commit_message>
<xml_diff>
--- a/assets/templates/clientes_template.xlsx
+++ b/assets/templates/clientes_template.xlsx
@@ -413,51 +413,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>codigo</t>
+          <t>cliente_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>nombre_fiscal</t>
+          <t>cliente_nombre_comercial</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>nombre_comercial</t>
+          <t>cliente_nombre_fiscal</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>contacto</t>
+          <t>cliente_nombre_interno</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>telefono</t>
+          <t>cliente_cif</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>cliente_telefono</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>direccion</t>
+          <t>cliente_email</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>notas</t>
+          <t>cliente_direccion</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
+        <is>
+          <t>cliente_direccion_cp</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cliente_direccion_localidad_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>cliente_direccion_municipio_id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>cliente_direccion_provincia_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>cliente_direccion_isla_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>cliente_tipo</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>cliente_grupo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>distribuidor_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
@@ -466,50 +506,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CLI-001</t>
+          <t>9c25da55-2eca-4288-a5f7-df337e8dd69f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Pan Ejemplo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Panaderia Ejemplo SL</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Pan Ejemplo</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ana Lopez</t>
+          <t>Pan Ejemplo Central</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>B12345678</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>600123123</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>compras@panejemplo.es</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Calle Mayor 1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Cliente piloto</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>35001</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>PANADERIA</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>si</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>